<commit_message>
Daily NSE scan: 2026-09-26
</commit_message>
<xml_diff>
--- a/output/2026-09-26/enriched_analysis.xlsx
+++ b/output/2026-09-26/enriched_analysis.xlsx
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>3.279</v>
+        <v>3.274</v>
       </c>
       <c r="W2" t="n">
-        <v>2928</v>
+        <v>2933</v>
       </c>
       <c r="X2" t="n">
-        <v>22.9</v>
+        <v>23</v>
       </c>
       <c r="Y2" t="n">
         <v>75</v>
@@ -1161,13 +1161,13 @@
         </is>
       </c>
       <c r="V3" t="n">
-        <v>0.824</v>
+        <v>0.8159999999999999</v>
       </c>
       <c r="W3" t="n">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="X3" t="n">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="Y3" t="n">
         <v>22</v>
@@ -1560,7 +1560,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
@@ -1568,7 +1568,7 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="F5" t="n">
         <v>19</v>
@@ -1623,13 +1623,13 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>0.998</v>
+        <v>1.003</v>
       </c>
       <c r="W5" t="n">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="X5" t="n">
-        <v>8.56</v>
+        <v>8.51</v>
       </c>
       <c r="Y5" t="n">
         <v>17</v>
@@ -1858,10 +1858,10 @@
         <v>0.052</v>
       </c>
       <c r="W6" t="n">
-        <v>2562</v>
+        <v>2561</v>
       </c>
       <c r="X6" t="n">
-        <v>8.81</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="Y6" t="n">
         <v>36</v>
@@ -2090,7 +2090,7 @@
         <v>0.121</v>
       </c>
       <c r="W7" t="n">
-        <v>2591</v>
+        <v>2594</v>
       </c>
       <c r="X7" t="n">
         <v>22.7</v>
@@ -2319,10 +2319,10 @@
         </is>
       </c>
       <c r="V8" t="n">
-        <v>0.446</v>
+        <v>0.445</v>
       </c>
       <c r="W8" t="n">
-        <v>2731</v>
+        <v>2736</v>
       </c>
       <c r="X8" t="n">
         <v>22.4</v>
@@ -2786,7 +2786,7 @@
         <v>0.048</v>
       </c>
       <c r="W10" t="n">
-        <v>1726</v>
+        <v>1722</v>
       </c>
       <c r="X10" t="n">
         <v>23.2</v>
@@ -3015,10 +3015,10 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>1.799</v>
+        <v>1.814</v>
       </c>
       <c r="W11" t="n">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="X11" t="inlineStr"/>
       <c r="Y11" t="n">
@@ -3248,7 +3248,7 @@
         <v>0.045</v>
       </c>
       <c r="W12" t="n">
-        <v>15946</v>
+        <v>15959</v>
       </c>
       <c r="X12" t="n">
         <v>40.6</v>
@@ -3477,13 +3477,13 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>0.392</v>
+        <v>0.388</v>
       </c>
       <c r="W13" t="n">
-        <v>1133</v>
+        <v>1143</v>
       </c>
       <c r="X13" t="n">
-        <v>57.7</v>
+        <v>58.2</v>
       </c>
       <c r="Y13" t="n">
         <v>21</v>
@@ -3709,13 +3709,13 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>2.316</v>
+        <v>2.325</v>
       </c>
       <c r="W14" t="n">
-        <v>2572</v>
+        <v>2563</v>
       </c>
       <c r="X14" t="n">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="Y14" t="n">
         <v>6</v>
@@ -4176,7 +4176,7 @@
         <v>0.07099999999999999</v>
       </c>
       <c r="W16" t="n">
-        <v>473</v>
+        <v>475</v>
       </c>
       <c r="X16" t="n">
         <v>14</v>
@@ -4637,10 +4637,10 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>0.043</v>
+        <v>0.042</v>
       </c>
       <c r="W18" t="n">
-        <v>704</v>
+        <v>705</v>
       </c>
       <c r="X18" t="n">
         <v>11.5</v>
@@ -4869,13 +4869,13 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>2.844</v>
+        <v>2.86</v>
       </c>
       <c r="W19" t="n">
-        <v>692</v>
+        <v>688</v>
       </c>
       <c r="X19" t="n">
-        <v>26</v>
+        <v>25.9</v>
       </c>
       <c r="Y19" t="n">
         <v>30</v>
@@ -5095,13 +5095,13 @@
         </is>
       </c>
       <c r="V20" t="n">
-        <v>0.623</v>
+        <v>0.624</v>
       </c>
       <c r="W20" t="n">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="X20" t="n">
-        <v>1215</v>
+        <v>1214</v>
       </c>
       <c r="Y20" t="n">
         <v>-61</v>
@@ -5323,13 +5323,13 @@
         </is>
       </c>
       <c r="V21" t="n">
-        <v>0.486</v>
+        <v>0.493</v>
       </c>
       <c r="W21" t="n">
-        <v>411</v>
+        <v>405</v>
       </c>
       <c r="X21" t="n">
-        <v>38.2</v>
+        <v>37.6</v>
       </c>
       <c r="Y21" t="n">
         <v>21</v>
@@ -5555,13 +5555,13 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>0.282</v>
+        <v>0.265</v>
       </c>
       <c r="W22" t="n">
-        <v>212</v>
+        <v>226</v>
       </c>
       <c r="X22" t="n">
-        <v>36.7</v>
+        <v>39.1</v>
       </c>
       <c r="Y22" t="n">
         <v>-44</v>
@@ -5790,10 +5790,10 @@
         <v>0.07099999999999999</v>
       </c>
       <c r="W23" t="n">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="X23" t="n">
-        <v>20.3</v>
+        <v>20.2</v>
       </c>
       <c r="Y23" t="n">
         <v>19</v>
@@ -6017,13 +6017,13 @@
         </is>
       </c>
       <c r="V24" t="n">
-        <v>0.163</v>
+        <v>0.162</v>
       </c>
       <c r="W24" t="n">
-        <v>679</v>
+        <v>686</v>
       </c>
       <c r="X24" t="n">
-        <v>56.7</v>
+        <v>57.3</v>
       </c>
       <c r="Y24" t="n">
         <v>3</v>
@@ -6252,7 +6252,7 @@
         <v>0.025</v>
       </c>
       <c r="W25" t="n">
-        <v>1002</v>
+        <v>999</v>
       </c>
       <c r="X25" t="inlineStr"/>
       <c r="Y25" t="n">
@@ -6482,7 +6482,7 @@
         <v>0.05</v>
       </c>
       <c r="W26" t="n">
-        <v>5251</v>
+        <v>5246</v>
       </c>
       <c r="X26" t="n">
         <v>34.2</v>
@@ -6946,7 +6946,7 @@
         <v>0.059</v>
       </c>
       <c r="W28" t="n">
-        <v>1872</v>
+        <v>1874</v>
       </c>
       <c r="X28" t="n">
         <v>43</v>
@@ -7175,13 +7175,13 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.137</v>
+        <v>0.135</v>
       </c>
       <c r="W29" t="n">
-        <v>363</v>
+        <v>368</v>
       </c>
       <c r="X29" t="n">
-        <v>5.86</v>
+        <v>5.93</v>
       </c>
       <c r="Y29" t="n">
         <v>118</v>
@@ -7406,7 +7406,7 @@
         <v>0.097</v>
       </c>
       <c r="W30" t="n">
-        <v>1532</v>
+        <v>1534</v>
       </c>
       <c r="X30" t="n">
         <v>13.9</v>
@@ -7635,13 +7635,13 @@
         </is>
       </c>
       <c r="V31" t="n">
-        <v>0.855</v>
+        <v>0.858</v>
       </c>
       <c r="W31" t="n">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="X31" t="n">
-        <v>6.79</v>
+        <v>6.75</v>
       </c>
       <c r="Y31" t="n">
         <v>31</v>
@@ -7863,10 +7863,10 @@
         </is>
       </c>
       <c r="V32" t="n">
-        <v>0.639</v>
+        <v>0.641</v>
       </c>
       <c r="W32" t="n">
-        <v>454</v>
+        <v>452</v>
       </c>
       <c r="X32" t="n">
         <v>11.3</v>
@@ -8098,7 +8098,7 @@
         <v>0.038</v>
       </c>
       <c r="W33" t="n">
-        <v>3497</v>
+        <v>3490</v>
       </c>
       <c r="X33" t="n">
         <v>20.7</v>
@@ -8330,10 +8330,10 @@
         <v>0</v>
       </c>
       <c r="W34" t="n">
-        <v>524</v>
+        <v>528</v>
       </c>
       <c r="X34" t="n">
-        <v>12.3</v>
+        <v>12.4</v>
       </c>
       <c r="Y34" t="n">
         <v>5</v>
@@ -8794,10 +8794,10 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W36" t="n">
-        <v>53396</v>
+        <v>53444</v>
       </c>
       <c r="X36" t="n">
-        <v>45.2</v>
+        <v>45.3</v>
       </c>
       <c r="Y36" t="n">
         <v>5</v>
@@ -9026,7 +9026,7 @@
         <v>0.02</v>
       </c>
       <c r="W37" t="n">
-        <v>9596</v>
+        <v>9589</v>
       </c>
       <c r="X37" t="n">
         <v>12.7</v>
@@ -9258,7 +9258,7 @@
         <v>0</v>
       </c>
       <c r="W38" t="n">
-        <v>3749</v>
+        <v>3748</v>
       </c>
       <c r="X38" t="n">
         <v>84.40000000000001</v>
@@ -9490,7 +9490,7 @@
         <v>0.008</v>
       </c>
       <c r="W39" t="n">
-        <v>5425</v>
+        <v>5427</v>
       </c>
       <c r="X39" t="n">
         <v>9.17</v>
@@ -10180,7 +10180,7 @@
         <v>0.129</v>
       </c>
       <c r="W42" t="n">
-        <v>577</v>
+        <v>578</v>
       </c>
       <c r="X42" t="n">
         <v>13.7</v>
@@ -10639,13 +10639,13 @@
         </is>
       </c>
       <c r="V44" t="n">
-        <v>0.269</v>
+        <v>0.272</v>
       </c>
       <c r="W44" t="n">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="X44" t="n">
-        <v>14.8</v>
+        <v>14.7</v>
       </c>
       <c r="Y44" t="n">
         <v>16</v>
@@ -10874,10 +10874,10 @@
         <v>0.233</v>
       </c>
       <c r="W45" t="n">
-        <v>969</v>
+        <v>966</v>
       </c>
       <c r="X45" t="n">
-        <v>26.4</v>
+        <v>26.3</v>
       </c>
       <c r="Y45" t="n">
         <v>9</v>
@@ -11106,7 +11106,7 @@
         <v>0.6870000000000001</v>
       </c>
       <c r="W46" t="n">
-        <v>3791</v>
+        <v>3789</v>
       </c>
       <c r="X46" t="n">
         <v>26.5</v>
@@ -11568,7 +11568,7 @@
         <v>0</v>
       </c>
       <c r="W48" t="n">
-        <v>8988</v>
+        <v>8983</v>
       </c>
       <c r="X48" t="n">
         <v>15.2</v>
@@ -11800,7 +11800,7 @@
         <v>0.224</v>
       </c>
       <c r="W49" t="n">
-        <v>1784</v>
+        <v>1785</v>
       </c>
       <c r="X49" t="n">
         <v>18.9</v>
@@ -12032,10 +12032,10 @@
         <v>0</v>
       </c>
       <c r="W50" t="n">
-        <v>119175</v>
+        <v>118820</v>
       </c>
       <c r="X50" t="n">
-        <v>34.3</v>
+        <v>34.2</v>
       </c>
       <c r="Y50" t="n">
         <v>18</v>
@@ -12261,13 +12261,13 @@
         </is>
       </c>
       <c r="V51" t="n">
-        <v>0.353</v>
+        <v>0.356</v>
       </c>
       <c r="W51" t="n">
-        <v>397</v>
+        <v>393</v>
       </c>
       <c r="X51" t="n">
-        <v>98.2</v>
+        <v>97.2</v>
       </c>
       <c r="Y51" t="n">
         <v>246</v>
@@ -12728,10 +12728,10 @@
         <v>0.043</v>
       </c>
       <c r="W53" t="n">
-        <v>1612</v>
+        <v>1613</v>
       </c>
       <c r="X53" t="n">
-        <v>21</v>
+        <v>21.1</v>
       </c>
       <c r="Y53" t="n">
         <v>10</v>
@@ -12960,7 +12960,7 @@
         <v>0.082</v>
       </c>
       <c r="W54" t="n">
-        <v>1670</v>
+        <v>1671</v>
       </c>
       <c r="X54" t="n">
         <v>30.2</v>

</xml_diff>